<commit_message>
Fix: Sync docs directory for GitHub Pages and add visible top-updated-at timestamp indicator
</commit_message>
<xml_diff>
--- a/docs/output/文中傳票維護匯入_全部合併_202610.xlsx
+++ b/docs/output/文中傳票維護匯入_全部合併_202610.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP13"/>
+  <dimension ref="A1:AP19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -856,7 +856,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>AR_一般顧客(月下) 營業收入</t>
+          <t>AR_一般顧客(隨意) 營業收入</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -872,7 +872,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>月宮(月下餐飲股份有限公司)</t>
+          <t>隨意小吃</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -895,14 +895,14 @@
         <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>17813</v>
+        <v>17196</v>
       </c>
       <c r="O3" t="n">
-        <v>17813</v>
+        <v>17196</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>AR_一般顧客(月下) 營業收入_銷貨收入</t>
+          <t>AR_一般顧客(隨意) 營業收入_銷貨收入</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr"/>
@@ -952,14 +952,14 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>4100-01</t>
+          <t>1130-01</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -987,14 +987,14 @@
         <v>1</v>
       </c>
       <c r="N4" t="n">
-        <v>17196</v>
+        <v>10820</v>
       </c>
       <c r="O4" t="n">
-        <v>17196</v>
+        <v>10820</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>AR_一般顧客(隨意) 營業收入_銷貨收入</t>
+          <t>AR_一般顧客(隨意) 營業收入_現金</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr"/>
@@ -1040,23 +1040,23 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>AR_一般顧客(月下) 營業收入</t>
+          <t>AR_一般顧客(隨意) 營業收入</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1130-01</t>
+          <t>1130-02</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>月宮(月下餐飲股份有限公司)</t>
+          <t>隨意小吃</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -1079,14 +1079,14 @@
         <v>1</v>
       </c>
       <c r="N5" t="n">
-        <v>6977</v>
+        <v>5210</v>
       </c>
       <c r="O5" t="n">
-        <v>6977</v>
+        <v>5210</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>AR_一般顧客(月下) 營業收入_現金</t>
+          <t>AR_一般顧客(隨意) 營業收入_linepay</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr"/>
@@ -1136,14 +1136,14 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>1130-01</t>
+          <t>1130-03</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1171,14 +1171,14 @@
         <v>1</v>
       </c>
       <c r="N6" t="n">
-        <v>10820</v>
+        <v>1740</v>
       </c>
       <c r="O6" t="n">
-        <v>10820</v>
+        <v>1740</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>AR_一般顧客(隨意) 營業收入_現金</t>
+          <t>AR_一般顧客(隨意) 營業收入_ubereats</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr"/>
@@ -1224,23 +1224,23 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>AR_一般顧客(月下) 營業收入</t>
+          <t>AR_一般顧客(隨意) 營業收入</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>1130-02</t>
+          <t>1130-04</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>月宮(月下餐飲股份有限公司)</t>
+          <t>隨意小吃</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -1263,14 +1263,14 @@
         <v>1</v>
       </c>
       <c r="N7" t="n">
-        <v>11038</v>
+        <v>286</v>
       </c>
       <c r="O7" t="n">
-        <v>11038</v>
+        <v>286</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>AR_一般顧客(月下) 營業收入_linepay</t>
+          <t>AR_一般顧客(隨意) 營業收入_foodpanda</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr"/>
@@ -1320,14 +1320,14 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>1130-02</t>
+          <t>2290</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1355,14 +1355,14 @@
         <v>1</v>
       </c>
       <c r="N8" t="n">
-        <v>5210</v>
+        <v>860</v>
       </c>
       <c r="O8" t="n">
-        <v>5210</v>
+        <v>860</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>AR_一般顧客(隨意) 營業收入_linepay</t>
+          <t>銷項AR_一般顧客(隨意) 銷項稅額</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr"/>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1412,14 +1412,14 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>1130-03</t>
+          <t>4100-01</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1447,14 +1447,14 @@
         <v>1</v>
       </c>
       <c r="N9" t="n">
-        <v>689</v>
+        <v>15463</v>
       </c>
       <c r="O9" t="n">
-        <v>689</v>
+        <v>15463</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>AR_一般顧客(月下) 營業收入_ubereats</t>
+          <t>AR_一般顧客(月下) 營業收入_銷貨收入</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr"/>
@@ -1495,7 +1495,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1504,14 +1504,14 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1130-03</t>
+          <t>4100-01</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1539,14 +1539,14 @@
         <v>1</v>
       </c>
       <c r="N10" t="n">
-        <v>1740</v>
+        <v>19232</v>
       </c>
       <c r="O10" t="n">
-        <v>1740</v>
+        <v>19232</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>AR_一般顧客(隨意) 營業收入_ubereats</t>
+          <t>AR_一般顧客(隨意) 營業收入_銷貨收入</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr"/>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1596,14 +1596,14 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2290</t>
+          <t>1130-01</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1631,14 +1631,14 @@
         <v>1</v>
       </c>
       <c r="N11" t="n">
-        <v>891</v>
+        <v>5728</v>
       </c>
       <c r="O11" t="n">
-        <v>891</v>
+        <v>5728</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>銷項AR_一般顧客(月下) 銷項稅額</t>
+          <t>AR_一般顧客(月下) 營業收入_現金</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr"/>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1688,14 +1688,14 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>1130-04</t>
+          <t>1130-01</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1723,14 +1723,14 @@
         <v>1</v>
       </c>
       <c r="N12" t="n">
-        <v>286</v>
+        <v>13890</v>
       </c>
       <c r="O12" t="n">
-        <v>286</v>
+        <v>13890</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>AR_一般顧客(隨意) 營業收入_foodpanda</t>
+          <t>AR_一般顧客(隨意) 營業收入_現金</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr"/>
@@ -1771,28 +1771,28 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>AR_一般顧客(隨意) 營業收入</t>
+          <t>AR_一般顧客(月下) 營業收入</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2290</t>
+          <t>1130-02</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>隨意小吃</t>
+          <t>月宮(月下餐飲股份有限公司)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -1815,14 +1815,14 @@
         <v>1</v>
       </c>
       <c r="N13" t="n">
-        <v>860</v>
+        <v>6498</v>
       </c>
       <c r="O13" t="n">
-        <v>860</v>
+        <v>6498</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>銷項AR_一般顧客(隨意) 銷項稅額</t>
+          <t>AR_一般顧客(月下) 營業收入_linepay</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr"/>
@@ -1852,6 +1852,558 @@
       <c r="AO13" t="inlineStr"/>
       <c r="AP13" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>@</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>AR_一般顧客(隨意) 營業收入</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>1130-02</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>隨意小吃</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>一般顧客</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>NTD</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>1</v>
+      </c>
+      <c r="N14" t="n">
+        <v>5970</v>
+      </c>
+      <c r="O14" t="n">
+        <v>5970</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>AR_一般顧客(隨意) 營業收入_linepay</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="inlineStr"/>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr"/>
+      <c r="AD14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr"/>
+      <c r="AG14" t="inlineStr"/>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
+      <c r="AJ14" t="inlineStr"/>
+      <c r="AK14" t="inlineStr"/>
+      <c r="AL14" t="inlineStr"/>
+      <c r="AM14" t="inlineStr"/>
+      <c r="AN14" t="inlineStr"/>
+      <c r="AO14" t="inlineStr"/>
+      <c r="AP14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>@</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>AR_一般顧客(月下) 營業收入</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>1130-03</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>月宮(月下餐飲股份有限公司)</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>一般顧客</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>NTD</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" t="n">
+        <v>1620</v>
+      </c>
+      <c r="O15" t="n">
+        <v>1620</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>AR_一般顧客(月下) 營業收入_ubereats</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="inlineStr"/>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
+      <c r="AD15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr"/>
+      <c r="AG15" t="inlineStr"/>
+      <c r="AH15" t="inlineStr"/>
+      <c r="AI15" t="inlineStr"/>
+      <c r="AJ15" t="inlineStr"/>
+      <c r="AK15" t="inlineStr"/>
+      <c r="AL15" t="inlineStr"/>
+      <c r="AM15" t="inlineStr"/>
+      <c r="AN15" t="inlineStr"/>
+      <c r="AO15" t="inlineStr"/>
+      <c r="AP15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>@</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>AR_一般顧客(隨意) 營業收入</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>1130-04</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>隨意小吃</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>一般顧客</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>NTD</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
+        <v>1</v>
+      </c>
+      <c r="N16" t="n">
+        <v>334</v>
+      </c>
+      <c r="O16" t="n">
+        <v>334</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>AR_一般顧客(隨意) 營業收入_foodpanda</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr"/>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="inlineStr"/>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
+      <c r="AD16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr"/>
+      <c r="AG16" t="inlineStr"/>
+      <c r="AH16" t="inlineStr"/>
+      <c r="AI16" t="inlineStr"/>
+      <c r="AJ16" t="inlineStr"/>
+      <c r="AK16" t="inlineStr"/>
+      <c r="AL16" t="inlineStr"/>
+      <c r="AM16" t="inlineStr"/>
+      <c r="AN16" t="inlineStr"/>
+      <c r="AO16" t="inlineStr"/>
+      <c r="AP16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>@</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>AR_一般顧客(月下) 營業收入</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>5</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>1130-05</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>月宮(月下餐飲股份有限公司)</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>一般顧客</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>NTD</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>1</v>
+      </c>
+      <c r="N17" t="n">
+        <v>2390</v>
+      </c>
+      <c r="O17" t="n">
+        <v>2390</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>AR_一般顧客(月下) 營業收入_偷訂</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr"/>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="inlineStr"/>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
+      <c r="AD17" t="inlineStr"/>
+      <c r="AE17" t="inlineStr"/>
+      <c r="AF17" t="inlineStr"/>
+      <c r="AG17" t="inlineStr"/>
+      <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr"/>
+      <c r="AJ17" t="inlineStr"/>
+      <c r="AK17" t="inlineStr"/>
+      <c r="AL17" t="inlineStr"/>
+      <c r="AM17" t="inlineStr"/>
+      <c r="AN17" t="inlineStr"/>
+      <c r="AO17" t="inlineStr"/>
+      <c r="AP17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>@</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>AR_一般顧客(隨意) 營業收入</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2290</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>隨意小吃</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>一般顧客</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>NTD</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>1</v>
+      </c>
+      <c r="N18" t="n">
+        <v>962</v>
+      </c>
+      <c r="O18" t="n">
+        <v>962</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>銷項AR_一般顧客(隨意) 銷項稅額</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
+      <c r="AA18" t="inlineStr"/>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
+      <c r="AD18" t="inlineStr"/>
+      <c r="AE18" t="inlineStr"/>
+      <c r="AF18" t="inlineStr"/>
+      <c r="AG18" t="inlineStr"/>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr"/>
+      <c r="AL18" t="inlineStr"/>
+      <c r="AM18" t="inlineStr"/>
+      <c r="AN18" t="inlineStr"/>
+      <c r="AO18" t="inlineStr"/>
+      <c r="AP18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>@</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>AR_一般顧客(月下) 營業收入</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>6</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2290</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>月宮(月下餐飲股份有限公司)</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>一般顧客</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>NTD</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N19" t="n">
+        <v>773</v>
+      </c>
+      <c r="O19" t="n">
+        <v>773</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>銷項AR_一般顧客(月下) 銷項稅額</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr"/>
+      <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
+      <c r="AA19" t="inlineStr"/>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
+      <c r="AD19" t="inlineStr"/>
+      <c r="AE19" t="inlineStr"/>
+      <c r="AF19" t="inlineStr"/>
+      <c r="AG19" t="inlineStr"/>
+      <c r="AH19" t="inlineStr"/>
+      <c r="AI19" t="inlineStr"/>
+      <c r="AJ19" t="inlineStr"/>
+      <c r="AK19" t="inlineStr"/>
+      <c r="AL19" t="inlineStr"/>
+      <c r="AM19" t="inlineStr"/>
+      <c r="AN19" t="inlineStr"/>
+      <c r="AO19" t="inlineStr"/>
+      <c r="AP19" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>